<commit_message>
Leaf area calculator: give the run line students use in the console
</commit_message>
<xml_diff>
--- a/leaf_area_calculator.xlsx
+++ b/leaf_area_calculator.xlsx
@@ -571,7 +571,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     python plot_lunchbox_photosynthesis.py --plant wheat --leaf_area 12 --save</t>
+          <t xml:space="preserve">     run ./plot_lunchbox_photosynthesis.py --plant wheat --leaf_area 12</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="B32" s="15">
-        <f>"python plot_lunchbox_photosynthesis.py --plant arabidopsis --leaf_area "&amp;E30&amp;" --save"</f>
+        <f>"run ./plot_lunchbox_photosynthesis.py --plant arabidopsis --leaf_area "&amp;E30</f>
         <v/>
       </c>
     </row>
@@ -1343,7 +1343,7 @@
         </is>
       </c>
       <c r="B32" s="15">
-        <f>"python plot_lunchbox_photosynthesis.py --plant wheat --leaf_area "&amp;E30&amp;" --save"</f>
+        <f>"run ./plot_lunchbox_photosynthesis.py --plant wheat --leaf_area "&amp;E30</f>
         <v/>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
         </is>
       </c>
       <c r="B32" s="15">
-        <f>"python plot_lunchbox_photosynthesis.py --plant maize --leaf_area "&amp;E30&amp;" --save"</f>
+        <f>"run ./plot_lunchbox_photosynthesis.py --plant maize --leaf_area "&amp;E30</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Use just --leaf_area in the run examples
--leaf_area overrides --plant, so giving both was confusing. --plant
is now only suggested for when the plant hasn't been measured.
</commit_message>
<xml_diff>
--- a/leaf_area_calculator.xlsx
+++ b/leaf_area_calculator.xlsx
@@ -571,7 +571,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     run ./plot_lunchbox_photosynthesis.py --plant wheat --leaf_area 12</t>
+          <t xml:space="preserve">     run ./plot_lunchbox_photosynthesis.py --leaf_area 12</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="B32" s="15">
-        <f>"run ./plot_lunchbox_photosynthesis.py --plant arabidopsis --leaf_area "&amp;E30</f>
+        <f>"run ./plot_lunchbox_photosynthesis.py --leaf_area "&amp;E30</f>
         <v/>
       </c>
     </row>
@@ -1343,7 +1343,7 @@
         </is>
       </c>
       <c r="B32" s="15">
-        <f>"run ./plot_lunchbox_photosynthesis.py --plant wheat --leaf_area "&amp;E30</f>
+        <f>"run ./plot_lunchbox_photosynthesis.py --leaf_area "&amp;E30</f>
         <v/>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
         </is>
       </c>
       <c r="B32" s="15">
-        <f>"run ./plot_lunchbox_photosynthesis.py --plant maize --leaf_area "&amp;E30</f>
+        <f>"run ./plot_lunchbox_photosynthesis.py --leaf_area "&amp;E30</f>
         <v/>
       </c>
     </row>

</xml_diff>